<commit_message>
docs(FCC-36-65): Strategy v2.1 — income+spending as Foundation layer + scenarios-not-predictions
Folds in the user's two notes after approving the v2.0 spine: (1) one rule reworded — we run
SCENARIOS for an intelligent estimate, never predict the future; (2) Income + spending now
explicit as the FOUNDATION layer (three layers: Foundation income/spending/accounts → Hero
investments/scenarios → Reassurance retirement), present+light in v1, more prominent as we
extend to 36-55. Superseded v1.0/v2.0 removed (in git history); README points to v2.1.
</commit_message>
<xml_diff>
--- a/docs/FCC-design-process-plan-v1.0-2026-06-29.xlsx
+++ b/docs/FCC-design-process-plan-v1.0-2026-06-29.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/palakjain/Vibe_Coding/finwise/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC555B0-F68E-A04D-BA83-567F6D055EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37667DC2-7C83-3D47-AED7-9366D216445E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="580" yWindow="4260" windowWidth="32100" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="580" yWindow="0" windowWidth="32100" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan &amp; approvals" sheetId="1" r:id="rId1"/>

</xml_diff>